<commit_message>
docs: update feedback Excel with gmail addresses
</commit_message>
<xml_diff>
--- a/docs/user_feedback.xlsx
+++ b/docs/user_feedback.xlsx
@@ -418,7 +418,7 @@
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -499,7 +499,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>amina.bello@email.com</t>
+          <t>aminabello@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>chukwu.emeka@email.com</t>
+          <t>chukwuemeka@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fatima.a@email.com</t>
+          <t>fatimaabubakar@gmail.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ibrahim.y@email.com</t>
+          <t>ibrahimyusuf@gmail.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>grace.o@email.com</t>
+          <t>graceokafor@gmail.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>oluwaseun.a@email.com</t>
+          <t>oluwaseunadeyemi@gmail.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>aisha.m@email.com</t>
+          <t>aishamohammed@gmail.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>emeka.n@email.com</t>
+          <t>emekanwosu@gmail.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>zainab.a@email.com</t>
+          <t>zainababdullahi@gmail.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tunde.b@email.com</t>
+          <t>tundebakare@gmail.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>

<commit_message>
docs: fix email format in feedback Excel - plain text, no mailto links
</commit_message>
<xml_diff>
--- a/docs/user_feedback.xlsx
+++ b/docs/user_feedback.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,7 +443,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>EMAIL ADRESS</t>
+          <t>EMAIL ADDRESS</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -497,7 +498,7 @@
           <t>Amina Bello</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>aminabello@gmail.com</t>
         </is>
@@ -552,7 +553,7 @@
           <t>Chukwu Emeka</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>chukwuemeka@gmail.com</t>
         </is>
@@ -607,7 +608,7 @@
           <t>Fatima Abubakar</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>fatimaabubakar@gmail.com</t>
         </is>
@@ -662,7 +663,7 @@
           <t>Ibrahim Yusuf</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>ibrahimyusuf@gmail.com</t>
         </is>
@@ -717,7 +718,7 @@
           <t>Grace Okafor</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>graceokafor@gmail.com</t>
         </is>
@@ -772,7 +773,7 @@
           <t>Oluwaseun Adeyemi</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>oluwaseunadeyemi@gmail.com</t>
         </is>
@@ -827,7 +828,7 @@
           <t>Aisha Mohammed</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>aishamohammed@gmail.com</t>
         </is>
@@ -882,7 +883,7 @@
           <t>Emeka Nwosu</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>emekanwosu@gmail.com</t>
         </is>
@@ -937,7 +938,7 @@
           <t>Zainab Abdullahi</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>zainababdullahi@gmail.com</t>
         </is>
@@ -992,7 +993,7 @@
           <t>Tunde Bakare</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>tundebakare@gmail.com</t>
         </is>

</xml_diff>

<commit_message>
docs: fix Excel - plain text emails, no hyperlinks, no mailto
</commit_message>
<xml_diff>
--- a/docs/user_feedback.xlsx
+++ b/docs/user_feedback.xlsx
@@ -17,13 +17,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -431,57 +436,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>FULL NAME</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>EMAIL ADDRESS</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>WALLET ADDRESS</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>NETWORK</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PRODUCT RATING</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>EASE OF USE</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>RELIABILITY</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>IMPROVEMENTS</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>RECOMMEND</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ADDITIONAL COMMENTS</t>
         </is>
@@ -498,12 +503,12 @@
           <t>Amina Bello</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>aminabello@gmail.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>GA2TSCRPPMJQDKHW5V47KTSGT5VFD3ZBKGUYCH4DU2OKXGE3NSOA7KCM</t>
         </is>
@@ -553,12 +558,12 @@
           <t>Chukwu Emeka</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>chukwuemeka@gmail.com</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>GAOPMTEEXOT7RXLGTA3CAIPLMXFRZWBPNPYJEP5MLHPPLVCP32L2VC5L</t>
         </is>
@@ -608,12 +613,12 @@
           <t>Fatima Abubakar</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>fatimaabubakar@gmail.com</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>GAFOWXXP5ME6AZMBVZAN2WPVWN7AWENT2VMQIXG6UUFEZ3SWN6L5Y3S2</t>
         </is>
@@ -663,12 +668,12 @@
           <t>Ibrahim Yusuf</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>ibrahimyusuf@gmail.com</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>GB626LQX3NAM5MHH43MFGZ3Z3P64EAQ6X5F4QXRKVZVSOF2LCA27BPOU</t>
         </is>
@@ -718,12 +723,12 @@
           <t>Grace Okafor</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>graceokafor@gmail.com</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>GA5O6CTG3HVN45WDASGIL5BQRGO5PFMZCOW4QLPJJTGFMMY4J4GKM3FC</t>
         </is>
@@ -773,12 +778,12 @@
           <t>Oluwaseun Adeyemi</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>oluwaseunadeyemi@gmail.com</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>GDPATR2J5I3TWHGKL656UBK4Y4MORBMDEZSR7TZFVYSXCX5V6QG4EMSH</t>
         </is>
@@ -828,12 +833,12 @@
           <t>Aisha Mohammed</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>aishamohammed@gmail.com</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>GAQVA7F24GHNNSGR5LNP7OAEBI55V3WG5KONOLKQLRQEBVBL4OP7V4OC</t>
         </is>
@@ -883,12 +888,12 @@
           <t>Emeka Nwosu</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>emekanwosu@gmail.com</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>GB5C3JFJN3FX2ZPTU2JJZYNCSLFYPRKAH72F5YEZUW2ZAYEGIQWHELPM</t>
         </is>
@@ -938,12 +943,12 @@
           <t>Zainab Abdullahi</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>zainababdullahi@gmail.com</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>GB4RV2TCOUM4MNU5IRQBB67Z2I65BXYUKI45ED6HIRUSQOD2EVP4QS55</t>
         </is>
@@ -993,12 +998,12 @@
           <t>Tunde Bakare</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>tundebakare@gmail.com</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>GAQOTCX43QCGKSQSFFUJ3J6P3SWHTDZ2UYANMBSFFBEWODCVGNNVW6CS</t>
         </is>

</xml_diff>